<commit_message>
tests pass before acceleration
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\08-ParallelSyncBoreholes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\08b-PreSim_ParallelSyncBoreholes\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E9DE16-1A47-48CC-AF33-E346AD55142C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F99AF09-6290-4AD2-AC93-BCAA86F290AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
     <sheet name="Ground" sheetId="2" r:id="rId2"/>
+    <sheet name="test" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>H [m]</t>
   </si>
@@ -77,6 +78,9 @@
   </si>
   <si>
     <t>0.1</t>
+  </si>
+  <si>
+    <t>The first 2 years should be given as historical load. The 3 year is the one simulated</t>
   </si>
 </sst>
 </file>
@@ -498,4 +502,22 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75E9FF2B-9005-48D7-B716-26E4F385D08F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="70.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added cusomised presim time from excel
</commit_message>
<xml_diff>
--- a/GeoInput.xlsx
+++ b/GeoInput.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TRNSYS18\TRNLib\CallingPython-Cffi\Examples\08b-PreSim_ParallelSyncBoreholes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5613532B-9F1E-49A0-BB51-FF7D6BAEA39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A929C75-2E80-4990-B8A9-B302C4C91F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Borehole" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>H [m]</t>
   </si>
@@ -47,9 +47,6 @@
     <t>rb</t>
   </si>
   <si>
-    <t>0.0575</t>
-  </si>
-  <si>
     <t>x</t>
   </si>
   <si>
@@ -62,24 +59,12 @@
     <t>k [W/mK]</t>
   </si>
   <si>
-    <t>3.1</t>
-  </si>
-  <si>
     <t>rho [kg/m3]</t>
   </si>
   <si>
     <t>cp[J/kg/k]</t>
   </si>
   <si>
-    <t>2300.0</t>
-  </si>
-  <si>
-    <t>870.0</t>
-  </si>
-  <si>
-    <t>0.1</t>
-  </si>
-  <si>
     <t>The first 2 years should be given as historical load. The 3 year is the one simulated</t>
   </si>
   <si>
@@ -87,6 +72,9 @@
   </si>
   <si>
     <t>Rb [mK/W]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presimulated steps </t>
   </si>
 </sst>
 </file>
@@ -410,13 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="7" width="8.7265625" style="1"/>
+    <col min="8" max="8" width="17.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -427,44 +417,50 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>100</v>
       </c>
       <c r="B2" s="2">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>3</v>
+      <c r="C2" s="2">
+        <v>5.7500000000000002E-2</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="H2" s="2">
+        <v>17520</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>100</v>
       </c>
       <c r="B3" s="2">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>13</v>
+      <c r="C3" s="2">
+        <v>5.7500000000000002E-2</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.1</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -484,30 +480,30 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
+      <c r="A2" s="2">
+        <v>3.1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>2300</v>
+      </c>
+      <c r="C2" s="2">
+        <v>870</v>
       </c>
       <c r="E2" s="2">
         <v>8</v>
@@ -532,7 +528,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>